<commit_message>
auto: update flight data
</commit_message>
<xml_diff>
--- a/flight_data/archive_flights.xlsx
+++ b/flight_data/archive_flights.xlsx
@@ -543,10 +543,14 @@
           <t>2355</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0014</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Gate Closed</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -559,7 +563,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -597,7 +601,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Departed</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -610,7 +614,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -648,7 +652,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Departed</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -661,7 +665,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -699,7 +703,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Departed</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -712,7 +716,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -750,7 +754,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Departed</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -763,7 +767,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -801,7 +805,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Departed</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
@@ -814,7 +818,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -852,7 +856,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Departed</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -865,7 +869,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -903,7 +907,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Gate Open</t>
+          <t>Departed</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -916,7 +920,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -954,7 +958,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Last Call</t>
+          <t>Departed</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -967,7 +971,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1002,10 +1006,14 @@
           <t>2230</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2300</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Last Call</t>
+          <t>Departed</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
@@ -1018,7 +1026,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1064,7 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Last Call</t>
+          <t>Departed</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
@@ -1069,7 +1077,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1115,7 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Last Call</t>
+          <t>Departed</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -1120,7 +1128,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1179,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1230,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1281,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1332,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1383,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1434,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1477,7 +1485,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1536,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1587,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1638,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1689,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1740,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1791,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1842,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1885,7 +1893,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1936,7 +1944,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1995,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2046,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2097,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2148,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2203,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2254,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2305,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2356,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2399,7 +2407,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2450,7 +2458,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2509,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2552,7 +2560,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2603,7 +2611,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2654,7 +2662,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2705,7 +2713,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2768,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2819,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2862,7 +2870,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2917,7 +2925,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -2972,7 +2980,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3031,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3074,7 +3082,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3133,7 @@
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3176,7 +3184,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3235,7 @@
       </c>
       <c r="M54" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3278,7 +3286,7 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3337,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3380,7 +3388,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3443,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3486,7 +3494,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3537,7 +3545,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3588,7 +3596,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3639,7 +3647,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3690,7 +3698,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3749,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3792,7 +3800,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3843,7 +3851,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3894,7 +3902,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3945,7 +3953,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -3996,7 +4004,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4059,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4102,7 +4110,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4153,7 +4161,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4204,7 +4212,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4255,7 +4263,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4310,7 +4318,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4361,7 +4369,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4412,7 +4420,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4463,7 +4471,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4514,7 +4522,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4565,7 +4573,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4616,7 +4624,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4675,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4718,7 +4726,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4773,7 +4781,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4824,7 +4832,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4879,7 +4887,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4930,7 +4938,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -4985,7 +4993,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>
@@ -5036,7 +5044,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>2026-05-11 18:28</t>
+          <t>2026-05-11 20:15</t>
         </is>
       </c>
     </row>

</xml_diff>